<commit_message>
Updated GHA_grids_kan10 model - 2026-06-18 23:22
</commit_message>
<xml_diff>
--- a/VerveStacks_GHA_grids_kan10/Sets-vervestacks.xlsx
+++ b/VerveStacks_GHA_grids_kan10/Sets-vervestacks.xlsx
@@ -5,16 +5,17 @@
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GHA_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8A8DA2-B584-4B0E-BD88-29945C98CFB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A51EB2C1-711F-4327-8652-34380D5C0C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
-    <sheet name="VEDA_Sets-Proc" sheetId="1" r:id="rId2"/>
+    <sheet name="geo_sets" sheetId="3" r:id="rId2"/>
+    <sheet name="VEDA_Sets-Proc" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="201">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -346,6 +347,300 @@
   </si>
   <si>
     <t>coal</t>
+  </si>
+  <si>
+    <t>~tfm_psets</t>
+  </si>
+  <si>
+    <t>setname</t>
+  </si>
+  <si>
+    <t>pset_co</t>
+  </si>
+  <si>
+    <t>pset_ci</t>
+  </si>
+  <si>
+    <t>t_pos_andor</t>
+  </si>
+  <si>
+    <t>p_w282578857-330_GHA</t>
+  </si>
+  <si>
+    <t>e_w282578857-330_GHA*</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
+    <t>p_w672526714-330_GHA</t>
+  </si>
+  <si>
+    <t>e_w672526714-330_GHA*</t>
+  </si>
+  <si>
+    <t>p_w674068904-225_GHA</t>
+  </si>
+  <si>
+    <t>e_w674068904-225_GHA*</t>
+  </si>
+  <si>
+    <t>p_w930744195-225_GHA</t>
+  </si>
+  <si>
+    <t>e_w930744195-225_GHA*</t>
+  </si>
+  <si>
+    <t>p_w1069597794-330_GHA</t>
+  </si>
+  <si>
+    <t>e_w1069597794-330_GHA*</t>
+  </si>
+  <si>
+    <t>p_w1155380911-330_GHA</t>
+  </si>
+  <si>
+    <t>e_w1155380911-330_GHA*</t>
+  </si>
+  <si>
+    <t>p_r15772152-330_GHA</t>
+  </si>
+  <si>
+    <t>e_r15772152-330_GHA*</t>
+  </si>
+  <si>
+    <t>p_GH1-225_GHA</t>
+  </si>
+  <si>
+    <t>e_GH1-225_GHA*</t>
+  </si>
+  <si>
+    <t>p_GH8-225_GHA</t>
+  </si>
+  <si>
+    <t>e_GH8-225_GHA*</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_001</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_001</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_002</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_002</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_003</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_003</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_004</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_004</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_005</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_005</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_006</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_006</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_007</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_007</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_008</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_008</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_009</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_009</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_010</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_010</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_011</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_011</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_012</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_012</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_013</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_013</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_014</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_014</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_015</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_015</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_016</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_016</t>
+  </si>
+  <si>
+    <t>rez_spv_GHA_017</t>
+  </si>
+  <si>
+    <t>elc_spv_GHA_017</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_001</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_001</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_002</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_002</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_003</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_003</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_004</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_004</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_005</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_005</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_006</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_006</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_007</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_007</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_008</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_008</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_009</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_009</t>
+  </si>
+  <si>
+    <t>rez_won_GHA_010</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_010</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_001</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_001</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_002</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_002</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_003</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_003</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_004</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_004</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_005</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_005</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_006</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_006</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_007</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_007</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_008</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_008</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_009</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_009</t>
+  </si>
+  <si>
+    <t>rez_wof_GHA_010</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_010</t>
   </si>
 </sst>
 </file>
@@ -1190,6 +1485,679 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3549D41A-7825-4F70-BDA6-6A093B5B6F6E}">
+  <dimension ref="B9:E56"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" t="s">
+        <v>112</v>
+      </c>
+      <c r="E12" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
+        <v>116</v>
+      </c>
+      <c r="E14" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B15" t="s">
+        <v>117</v>
+      </c>
+      <c r="C15" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" t="s">
+        <v>118</v>
+      </c>
+      <c r="E15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B16" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B17" t="s">
+        <v>121</v>
+      </c>
+      <c r="C17" t="s">
+        <v>122</v>
+      </c>
+      <c r="D17" t="s">
+        <v>122</v>
+      </c>
+      <c r="E17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B18" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" t="s">
+        <v>124</v>
+      </c>
+      <c r="E18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" t="s">
+        <v>126</v>
+      </c>
+      <c r="D19" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B20" t="s">
+        <v>127</v>
+      </c>
+      <c r="C20" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" t="s">
+        <v>128</v>
+      </c>
+      <c r="E20" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" t="s">
+        <v>130</v>
+      </c>
+      <c r="D21" t="s">
+        <v>130</v>
+      </c>
+      <c r="E21" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B22" t="s">
+        <v>131</v>
+      </c>
+      <c r="C22" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" t="s">
+        <v>132</v>
+      </c>
+      <c r="E22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B23" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" t="s">
+        <v>134</v>
+      </c>
+      <c r="D23" t="s">
+        <v>134</v>
+      </c>
+      <c r="E23" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B24" t="s">
+        <v>135</v>
+      </c>
+      <c r="C24" t="s">
+        <v>136</v>
+      </c>
+      <c r="D24" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B25" t="s">
+        <v>137</v>
+      </c>
+      <c r="C25" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25" t="s">
+        <v>138</v>
+      </c>
+      <c r="E25" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B26" t="s">
+        <v>139</v>
+      </c>
+      <c r="C26" t="s">
+        <v>140</v>
+      </c>
+      <c r="D26" t="s">
+        <v>140</v>
+      </c>
+      <c r="E26" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B27" t="s">
+        <v>141</v>
+      </c>
+      <c r="C27" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" t="s">
+        <v>142</v>
+      </c>
+      <c r="E27" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B28" t="s">
+        <v>143</v>
+      </c>
+      <c r="C28" t="s">
+        <v>144</v>
+      </c>
+      <c r="D28" t="s">
+        <v>144</v>
+      </c>
+      <c r="E28" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B29" t="s">
+        <v>145</v>
+      </c>
+      <c r="C29" t="s">
+        <v>146</v>
+      </c>
+      <c r="D29" t="s">
+        <v>146</v>
+      </c>
+      <c r="E29" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B30" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" t="s">
+        <v>148</v>
+      </c>
+      <c r="D30" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C31" t="s">
+        <v>150</v>
+      </c>
+      <c r="D31" t="s">
+        <v>150</v>
+      </c>
+      <c r="E31" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B32" t="s">
+        <v>151</v>
+      </c>
+      <c r="C32" t="s">
+        <v>152</v>
+      </c>
+      <c r="D32" t="s">
+        <v>152</v>
+      </c>
+      <c r="E32" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B33" t="s">
+        <v>153</v>
+      </c>
+      <c r="C33" t="s">
+        <v>154</v>
+      </c>
+      <c r="D33" t="s">
+        <v>154</v>
+      </c>
+      <c r="E33" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B34" t="s">
+        <v>155</v>
+      </c>
+      <c r="C34" t="s">
+        <v>156</v>
+      </c>
+      <c r="D34" t="s">
+        <v>156</v>
+      </c>
+      <c r="E34" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B35" t="s">
+        <v>157</v>
+      </c>
+      <c r="C35" t="s">
+        <v>158</v>
+      </c>
+      <c r="D35" t="s">
+        <v>158</v>
+      </c>
+      <c r="E35" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B36" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" t="s">
+        <v>160</v>
+      </c>
+      <c r="D36" t="s">
+        <v>160</v>
+      </c>
+      <c r="E36" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B37" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" t="s">
+        <v>162</v>
+      </c>
+      <c r="D37" t="s">
+        <v>162</v>
+      </c>
+      <c r="E37" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B38" t="s">
+        <v>163</v>
+      </c>
+      <c r="C38" t="s">
+        <v>164</v>
+      </c>
+      <c r="D38" t="s">
+        <v>164</v>
+      </c>
+      <c r="E38" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B39" t="s">
+        <v>165</v>
+      </c>
+      <c r="C39" t="s">
+        <v>166</v>
+      </c>
+      <c r="D39" t="s">
+        <v>166</v>
+      </c>
+      <c r="E39" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B40" t="s">
+        <v>167</v>
+      </c>
+      <c r="C40" t="s">
+        <v>168</v>
+      </c>
+      <c r="D40" t="s">
+        <v>168</v>
+      </c>
+      <c r="E40" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B41" t="s">
+        <v>169</v>
+      </c>
+      <c r="C41" t="s">
+        <v>170</v>
+      </c>
+      <c r="D41" t="s">
+        <v>170</v>
+      </c>
+      <c r="E41" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B42" t="s">
+        <v>171</v>
+      </c>
+      <c r="C42" t="s">
+        <v>172</v>
+      </c>
+      <c r="D42" t="s">
+        <v>172</v>
+      </c>
+      <c r="E42" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B43" t="s">
+        <v>173</v>
+      </c>
+      <c r="C43" t="s">
+        <v>174</v>
+      </c>
+      <c r="D43" t="s">
+        <v>174</v>
+      </c>
+      <c r="E43" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B44" t="s">
+        <v>175</v>
+      </c>
+      <c r="C44" t="s">
+        <v>176</v>
+      </c>
+      <c r="D44" t="s">
+        <v>176</v>
+      </c>
+      <c r="E44" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B45" t="s">
+        <v>177</v>
+      </c>
+      <c r="C45" t="s">
+        <v>178</v>
+      </c>
+      <c r="D45" t="s">
+        <v>178</v>
+      </c>
+      <c r="E45" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B46" t="s">
+        <v>179</v>
+      </c>
+      <c r="C46" t="s">
+        <v>180</v>
+      </c>
+      <c r="D46" t="s">
+        <v>180</v>
+      </c>
+      <c r="E46" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B47" t="s">
+        <v>181</v>
+      </c>
+      <c r="C47" t="s">
+        <v>182</v>
+      </c>
+      <c r="D47" t="s">
+        <v>182</v>
+      </c>
+      <c r="E47" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B48" t="s">
+        <v>183</v>
+      </c>
+      <c r="C48" t="s">
+        <v>184</v>
+      </c>
+      <c r="D48" t="s">
+        <v>184</v>
+      </c>
+      <c r="E48" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B49" t="s">
+        <v>185</v>
+      </c>
+      <c r="C49" t="s">
+        <v>186</v>
+      </c>
+      <c r="D49" t="s">
+        <v>186</v>
+      </c>
+      <c r="E49" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B50" t="s">
+        <v>187</v>
+      </c>
+      <c r="C50" t="s">
+        <v>188</v>
+      </c>
+      <c r="D50" t="s">
+        <v>188</v>
+      </c>
+      <c r="E50" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B51" t="s">
+        <v>189</v>
+      </c>
+      <c r="C51" t="s">
+        <v>190</v>
+      </c>
+      <c r="D51" t="s">
+        <v>190</v>
+      </c>
+      <c r="E51" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B52" t="s">
+        <v>191</v>
+      </c>
+      <c r="C52" t="s">
+        <v>192</v>
+      </c>
+      <c r="D52" t="s">
+        <v>192</v>
+      </c>
+      <c r="E52" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B53" t="s">
+        <v>193</v>
+      </c>
+      <c r="C53" t="s">
+        <v>194</v>
+      </c>
+      <c r="D53" t="s">
+        <v>194</v>
+      </c>
+      <c r="E53" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B54" t="s">
+        <v>195</v>
+      </c>
+      <c r="C54" t="s">
+        <v>196</v>
+      </c>
+      <c r="D54" t="s">
+        <v>196</v>
+      </c>
+      <c r="E54" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B55" t="s">
+        <v>197</v>
+      </c>
+      <c r="C55" t="s">
+        <v>198</v>
+      </c>
+      <c r="D55" t="s">
+        <v>198</v>
+      </c>
+      <c r="E55" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B56" t="s">
+        <v>199</v>
+      </c>
+      <c r="C56" t="s">
+        <v>200</v>
+      </c>
+      <c r="D56" t="s">
+        <v>200</v>
+      </c>
+      <c r="E56" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
   <dimension ref="A1:K34"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>